<commit_message>
M6-M8 (pre-reveal parts): Mack, bootstraps, sensitivities, illustrative LIC, one-year simulation
Uses upper-triangle data only (no holdout read). Custom selected-reserve bootstrap: mean 362,962, CV 6.3%.
Illustrative net LIC 375,224 (BE 360,568 + RA75 14,656). One-year 99.5% L / BE 12.0% vs 27% standard formula.
Calibration, back-tests and the one-year back-test wait for the selection-locked tag.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/reserving_check.xlsx
+++ b/excel/reserving_check.xlsx
@@ -7,12 +7,13 @@
   </bookViews>
   <sheets>
     <sheet name="check" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="mack" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t xml:space="preserve">Reserving check - NAIC 1767 - paid, USD thousands, as at 2007-12-31 (US commercial auto, net, NAIC Schedule P)</t>
   </si>
@@ -96,6 +97,30 @@
   </si>
   <si>
     <t xml:space="preserve">ELR_CapeCod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mack (1993) total standard error, paid, all-year volume-weighted factors, no tail (USD thousands)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sigma2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completed triangle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">msep_i</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cross_i</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Mack SE</t>
   </si>
 </sst>
 </file>
@@ -1207,4 +1232,795 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B4" t="n">
+        <v>52793</v>
+      </c>
+      <c r="C4" t="n">
+        <v>93473</v>
+      </c>
+      <c r="D4" t="n">
+        <v>122582</v>
+      </c>
+      <c r="E4" t="n">
+        <v>138893</v>
+      </c>
+      <c r="F4" t="n">
+        <v>148204</v>
+      </c>
+      <c r="G4" t="n">
+        <v>152388</v>
+      </c>
+      <c r="H4" t="n">
+        <v>154182</v>
+      </c>
+      <c r="I4" t="n">
+        <v>156195</v>
+      </c>
+      <c r="J4" t="n">
+        <v>157619</v>
+      </c>
+      <c r="K4" t="n">
+        <v>157992</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B5" t="n">
+        <v>54899</v>
+      </c>
+      <c r="C5" t="n">
+        <v>94758</v>
+      </c>
+      <c r="D5" t="n">
+        <v>124791</v>
+      </c>
+      <c r="E5" t="n">
+        <v>140829</v>
+      </c>
+      <c r="F5" t="n">
+        <v>150092</v>
+      </c>
+      <c r="G5" t="n">
+        <v>153731</v>
+      </c>
+      <c r="H5" t="n">
+        <v>155795</v>
+      </c>
+      <c r="I5" t="n">
+        <v>157759</v>
+      </c>
+      <c r="J5" t="n">
+        <v>158417</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B6" t="n">
+        <v>55038</v>
+      </c>
+      <c r="C6" t="n">
+        <v>102876</v>
+      </c>
+      <c r="D6" t="n">
+        <v>133577</v>
+      </c>
+      <c r="E6" t="n">
+        <v>151644</v>
+      </c>
+      <c r="F6" t="n">
+        <v>161995</v>
+      </c>
+      <c r="G6" t="n">
+        <v>167149</v>
+      </c>
+      <c r="H6" t="n">
+        <v>170113</v>
+      </c>
+      <c r="I6" t="n">
+        <v>170731</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B7" t="n">
+        <v>55821</v>
+      </c>
+      <c r="C7" t="n">
+        <v>95917</v>
+      </c>
+      <c r="D7" t="n">
+        <v>119685</v>
+      </c>
+      <c r="E7" t="n">
+        <v>134023</v>
+      </c>
+      <c r="F7" t="n">
+        <v>142762</v>
+      </c>
+      <c r="G7" t="n">
+        <v>147893</v>
+      </c>
+      <c r="H7" t="n">
+        <v>149899</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B8" t="n">
+        <v>59699</v>
+      </c>
+      <c r="C8" t="n">
+        <v>106467</v>
+      </c>
+      <c r="D8" t="n">
+        <v>135085</v>
+      </c>
+      <c r="E8" t="n">
+        <v>156412</v>
+      </c>
+      <c r="F8" t="n">
+        <v>168340</v>
+      </c>
+      <c r="G8" t="n">
+        <v>173788</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B9" t="n">
+        <v>61023</v>
+      </c>
+      <c r="C9" t="n">
+        <v>108021</v>
+      </c>
+      <c r="D9" t="n">
+        <v>136734</v>
+      </c>
+      <c r="E9" t="n">
+        <v>159422</v>
+      </c>
+      <c r="F9" t="n">
+        <v>173331</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B10" t="n">
+        <v>56934</v>
+      </c>
+      <c r="C10" t="n">
+        <v>104545</v>
+      </c>
+      <c r="D10" t="n">
+        <v>134687</v>
+      </c>
+      <c r="E10" t="n">
+        <v>159177</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B11" t="n">
+        <v>64679</v>
+      </c>
+      <c r="C11" t="n">
+        <v>119626</v>
+      </c>
+      <c r="D11" t="n">
+        <v>167302</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B12" t="n">
+        <v>75287</v>
+      </c>
+      <c r="C12" t="n">
+        <v>126104</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B13" t="n">
+        <v>74744</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" t="str">
+        <f>SUM(C4:C12)/SUM(B4:B12)</f>
+      </c>
+      <c r="C15" t="str">
+        <f>SUM(D4:D11)/SUM(C4:C11)</f>
+      </c>
+      <c r="D15" t="str">
+        <f>SUM(E4:E10)/SUM(D4:D10)</f>
+      </c>
+      <c r="E15" t="str">
+        <f>SUM(F4:F9)/SUM(E4:E9)</f>
+      </c>
+      <c r="F15" t="str">
+        <f>SUM(G4:G8)/SUM(F4:F8)</f>
+      </c>
+      <c r="G15" t="str">
+        <f>SUM(H4:H7)/SUM(G4:G7)</f>
+      </c>
+      <c r="H15" t="str">
+        <f>SUM(I4:I6)/SUM(H4:H6)</f>
+      </c>
+      <c r="I15" t="str">
+        <f>SUM(J4:J5)/SUM(I4:I5)</f>
+      </c>
+      <c r="J15" t="str">
+        <f>SUM(K4:K4)/SUM(J4:J4)</f>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="str">
+        <f>SUMPRODUCT(B4:B12,(C4:C12/B4:B12-B15)^2)/(9-1)</f>
+      </c>
+      <c r="C16" t="str">
+        <f>SUMPRODUCT(C4:C11,(D4:D11/C4:C11-C15)^2)/(8-1)</f>
+      </c>
+      <c r="D16" t="str">
+        <f>SUMPRODUCT(D4:D10,(E4:E10/D4:D10-D15)^2)/(7-1)</f>
+      </c>
+      <c r="E16" t="str">
+        <f>SUMPRODUCT(E4:E9,(F4:F9/E4:E9-E15)^2)/(6-1)</f>
+      </c>
+      <c r="F16" t="str">
+        <f>SUMPRODUCT(F4:F8,(G4:G8/F4:F8-F15)^2)/(5-1)</f>
+      </c>
+      <c r="G16" t="str">
+        <f>SUMPRODUCT(G4:G7,(H4:H7/G4:G7-G15)^2)/(4-1)</f>
+      </c>
+      <c r="H16" t="str">
+        <f>SUMPRODUCT(H4:H6,(I4:I6/H4:H6-H15)^2)/(3-1)</f>
+      </c>
+      <c r="I16" t="str">
+        <f>SUMPRODUCT(I4:I5,(J4:J5/I4:I5-I15)^2)/(2-1)</f>
+      </c>
+      <c r="J16" t="str">
+        <f>MIN(I16^2/H16,H16,I16)</f>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" t="str">
+        <f>SUM(B4:B12)</f>
+      </c>
+      <c r="C17" t="str">
+        <f>SUM(C4:C11)</f>
+      </c>
+      <c r="D17" t="str">
+        <f>SUM(D4:D10)</f>
+      </c>
+      <c r="E17" t="str">
+        <f>SUM(E4:E9)</f>
+      </c>
+      <c r="F17" t="str">
+        <f>SUM(F4:F8)</f>
+      </c>
+      <c r="G17" t="str">
+        <f>SUM(G4:G7)</f>
+      </c>
+      <c r="H17" t="str">
+        <f>SUM(H4:H6)</f>
+      </c>
+      <c r="I17" t="str">
+        <f>SUM(I4:I5)</f>
+      </c>
+      <c r="J17" t="str">
+        <f>SUM(J4:J4)</f>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="M19" t="s">
+        <v>33</v>
+      </c>
+      <c r="N19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <f>A4</f>
+      </c>
+      <c r="B20" t="str">
+        <f>B4</f>
+      </c>
+      <c r="C20" t="str">
+        <f>C4</f>
+      </c>
+      <c r="D20" t="str">
+        <f>D4</f>
+      </c>
+      <c r="E20" t="str">
+        <f>E4</f>
+      </c>
+      <c r="F20" t="str">
+        <f>F4</f>
+      </c>
+      <c r="G20" t="str">
+        <f>G4</f>
+      </c>
+      <c r="H20" t="str">
+        <f>H4</f>
+      </c>
+      <c r="I20" t="str">
+        <f>I4</f>
+      </c>
+      <c r="J20" t="str">
+        <f>J4</f>
+      </c>
+      <c r="K20" t="str">
+        <f>K4</f>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <f>A5</f>
+      </c>
+      <c r="B21" t="str">
+        <f>B5</f>
+      </c>
+      <c r="C21" t="str">
+        <f>C5</f>
+      </c>
+      <c r="D21" t="str">
+        <f>D5</f>
+      </c>
+      <c r="E21" t="str">
+        <f>E5</f>
+      </c>
+      <c r="F21" t="str">
+        <f>F5</f>
+      </c>
+      <c r="G21" t="str">
+        <f>G5</f>
+      </c>
+      <c r="H21" t="str">
+        <f>H5</f>
+      </c>
+      <c r="I21" t="str">
+        <f>I5</f>
+      </c>
+      <c r="J21" t="str">
+        <f>J5</f>
+      </c>
+      <c r="K21" t="str">
+        <f>J21*J15</f>
+      </c>
+      <c r="M21" t="str">
+        <f>K21^2*SUMPRODUCT(J$16:J$16/J$15:J$15^2,1/J21:J21+1/J$17:J$17)</f>
+      </c>
+      <c r="N21" t="str">
+        <f>K21*SUM(K22:K29)*SUMPRODUCT(2*J$16:J$16/J$15:J$15^2/J$17:J$17)</f>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <f>A6</f>
+      </c>
+      <c r="B22" t="str">
+        <f>B6</f>
+      </c>
+      <c r="C22" t="str">
+        <f>C6</f>
+      </c>
+      <c r="D22" t="str">
+        <f>D6</f>
+      </c>
+      <c r="E22" t="str">
+        <f>E6</f>
+      </c>
+      <c r="F22" t="str">
+        <f>F6</f>
+      </c>
+      <c r="G22" t="str">
+        <f>G6</f>
+      </c>
+      <c r="H22" t="str">
+        <f>H6</f>
+      </c>
+      <c r="I22" t="str">
+        <f>I6</f>
+      </c>
+      <c r="J22" t="str">
+        <f>I22*I15</f>
+      </c>
+      <c r="K22" t="str">
+        <f>J22*J15</f>
+      </c>
+      <c r="M22" t="str">
+        <f>K22^2*SUMPRODUCT(I$16:J$16/I$15:J$15^2,1/I22:J22+1/I$17:J$17)</f>
+      </c>
+      <c r="N22" t="str">
+        <f>K22*SUM(K23:K29)*SUMPRODUCT(2*I$16:J$16/I$15:J$15^2/I$17:J$17)</f>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <f>A7</f>
+      </c>
+      <c r="B23" t="str">
+        <f>B7</f>
+      </c>
+      <c r="C23" t="str">
+        <f>C7</f>
+      </c>
+      <c r="D23" t="str">
+        <f>D7</f>
+      </c>
+      <c r="E23" t="str">
+        <f>E7</f>
+      </c>
+      <c r="F23" t="str">
+        <f>F7</f>
+      </c>
+      <c r="G23" t="str">
+        <f>G7</f>
+      </c>
+      <c r="H23" t="str">
+        <f>H7</f>
+      </c>
+      <c r="I23" t="str">
+        <f>H23*H15</f>
+      </c>
+      <c r="J23" t="str">
+        <f>I23*I15</f>
+      </c>
+      <c r="K23" t="str">
+        <f>J23*J15</f>
+      </c>
+      <c r="M23" t="str">
+        <f>K23^2*SUMPRODUCT(H$16:J$16/H$15:J$15^2,1/H23:J23+1/H$17:J$17)</f>
+      </c>
+      <c r="N23" t="str">
+        <f>K23*SUM(K24:K29)*SUMPRODUCT(2*H$16:J$16/H$15:J$15^2/H$17:J$17)</f>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <f>A8</f>
+      </c>
+      <c r="B24" t="str">
+        <f>B8</f>
+      </c>
+      <c r="C24" t="str">
+        <f>C8</f>
+      </c>
+      <c r="D24" t="str">
+        <f>D8</f>
+      </c>
+      <c r="E24" t="str">
+        <f>E8</f>
+      </c>
+      <c r="F24" t="str">
+        <f>F8</f>
+      </c>
+      <c r="G24" t="str">
+        <f>G8</f>
+      </c>
+      <c r="H24" t="str">
+        <f>G24*G15</f>
+      </c>
+      <c r="I24" t="str">
+        <f>H24*H15</f>
+      </c>
+      <c r="J24" t="str">
+        <f>I24*I15</f>
+      </c>
+      <c r="K24" t="str">
+        <f>J24*J15</f>
+      </c>
+      <c r="M24" t="str">
+        <f>K24^2*SUMPRODUCT(G$16:J$16/G$15:J$15^2,1/G24:J24+1/G$17:J$17)</f>
+      </c>
+      <c r="N24" t="str">
+        <f>K24*SUM(K25:K29)*SUMPRODUCT(2*G$16:J$16/G$15:J$15^2/G$17:J$17)</f>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <f>A9</f>
+      </c>
+      <c r="B25" t="str">
+        <f>B9</f>
+      </c>
+      <c r="C25" t="str">
+        <f>C9</f>
+      </c>
+      <c r="D25" t="str">
+        <f>D9</f>
+      </c>
+      <c r="E25" t="str">
+        <f>E9</f>
+      </c>
+      <c r="F25" t="str">
+        <f>F9</f>
+      </c>
+      <c r="G25" t="str">
+        <f>F25*F15</f>
+      </c>
+      <c r="H25" t="str">
+        <f>G25*G15</f>
+      </c>
+      <c r="I25" t="str">
+        <f>H25*H15</f>
+      </c>
+      <c r="J25" t="str">
+        <f>I25*I15</f>
+      </c>
+      <c r="K25" t="str">
+        <f>J25*J15</f>
+      </c>
+      <c r="M25" t="str">
+        <f>K25^2*SUMPRODUCT(F$16:J$16/F$15:J$15^2,1/F25:J25+1/F$17:J$17)</f>
+      </c>
+      <c r="N25" t="str">
+        <f>K25*SUM(K26:K29)*SUMPRODUCT(2*F$16:J$16/F$15:J$15^2/F$17:J$17)</f>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <f>A10</f>
+      </c>
+      <c r="B26" t="str">
+        <f>B10</f>
+      </c>
+      <c r="C26" t="str">
+        <f>C10</f>
+      </c>
+      <c r="D26" t="str">
+        <f>D10</f>
+      </c>
+      <c r="E26" t="str">
+        <f>E10</f>
+      </c>
+      <c r="F26" t="str">
+        <f>E26*E15</f>
+      </c>
+      <c r="G26" t="str">
+        <f>F26*F15</f>
+      </c>
+      <c r="H26" t="str">
+        <f>G26*G15</f>
+      </c>
+      <c r="I26" t="str">
+        <f>H26*H15</f>
+      </c>
+      <c r="J26" t="str">
+        <f>I26*I15</f>
+      </c>
+      <c r="K26" t="str">
+        <f>J26*J15</f>
+      </c>
+      <c r="M26" t="str">
+        <f>K26^2*SUMPRODUCT(E$16:J$16/E$15:J$15^2,1/E26:J26+1/E$17:J$17)</f>
+      </c>
+      <c r="N26" t="str">
+        <f>K26*SUM(K27:K29)*SUMPRODUCT(2*E$16:J$16/E$15:J$15^2/E$17:J$17)</f>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <f>A11</f>
+      </c>
+      <c r="B27" t="str">
+        <f>B11</f>
+      </c>
+      <c r="C27" t="str">
+        <f>C11</f>
+      </c>
+      <c r="D27" t="str">
+        <f>D11</f>
+      </c>
+      <c r="E27" t="str">
+        <f>D27*D15</f>
+      </c>
+      <c r="F27" t="str">
+        <f>E27*E15</f>
+      </c>
+      <c r="G27" t="str">
+        <f>F27*F15</f>
+      </c>
+      <c r="H27" t="str">
+        <f>G27*G15</f>
+      </c>
+      <c r="I27" t="str">
+        <f>H27*H15</f>
+      </c>
+      <c r="J27" t="str">
+        <f>I27*I15</f>
+      </c>
+      <c r="K27" t="str">
+        <f>J27*J15</f>
+      </c>
+      <c r="M27" t="str">
+        <f>K27^2*SUMPRODUCT(D$16:J$16/D$15:J$15^2,1/D27:J27+1/D$17:J$17)</f>
+      </c>
+      <c r="N27" t="str">
+        <f>K27*SUM(K28:K29)*SUMPRODUCT(2*D$16:J$16/D$15:J$15^2/D$17:J$17)</f>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <f>A12</f>
+      </c>
+      <c r="B28" t="str">
+        <f>B12</f>
+      </c>
+      <c r="C28" t="str">
+        <f>C12</f>
+      </c>
+      <c r="D28" t="str">
+        <f>C28*C15</f>
+      </c>
+      <c r="E28" t="str">
+        <f>D28*D15</f>
+      </c>
+      <c r="F28" t="str">
+        <f>E28*E15</f>
+      </c>
+      <c r="G28" t="str">
+        <f>F28*F15</f>
+      </c>
+      <c r="H28" t="str">
+        <f>G28*G15</f>
+      </c>
+      <c r="I28" t="str">
+        <f>H28*H15</f>
+      </c>
+      <c r="J28" t="str">
+        <f>I28*I15</f>
+      </c>
+      <c r="K28" t="str">
+        <f>J28*J15</f>
+      </c>
+      <c r="M28" t="str">
+        <f>K28^2*SUMPRODUCT(C$16:J$16/C$15:J$15^2,1/C28:J28+1/C$17:J$17)</f>
+      </c>
+      <c r="N28" t="str">
+        <f>K28*SUM(K29:K29)*SUMPRODUCT(2*C$16:J$16/C$15:J$15^2/C$17:J$17)</f>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <f>A13</f>
+      </c>
+      <c r="B29" t="str">
+        <f>B13</f>
+      </c>
+      <c r="C29" t="str">
+        <f>B29*B15</f>
+      </c>
+      <c r="D29" t="str">
+        <f>C29*C15</f>
+      </c>
+      <c r="E29" t="str">
+        <f>D29*D15</f>
+      </c>
+      <c r="F29" t="str">
+        <f>E29*E15</f>
+      </c>
+      <c r="G29" t="str">
+        <f>F29*F15</f>
+      </c>
+      <c r="H29" t="str">
+        <f>G29*G15</f>
+      </c>
+      <c r="I29" t="str">
+        <f>H29*H15</f>
+      </c>
+      <c r="J29" t="str">
+        <f>I29*I15</f>
+      </c>
+      <c r="K29" t="str">
+        <f>J29*J15</f>
+      </c>
+      <c r="M29" t="str">
+        <f>K29^2*SUMPRODUCT(B$16:J$16/B$15:J$15^2,1/B29:J29+1/B$17:J$17)</f>
+      </c>
+      <c r="N29" t="str">
+        <f>K29*0*SUMPRODUCT(2*B$16:J$16/B$15:J$15^2/B$17:J$17)</f>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" t="str">
+        <f>SQRT(SUM(M20:M29)+SUM(N20:N29))</f>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>